<commit_message>
Fix fidelity dashboard gaps for Cancer PCA corr and Mean Error Pct.
</commit_message>
<xml_diff>
--- a/paper results/1. Cancer/fidelity_privacy_metrics.xlsx
+++ b/paper results/1. Cancer/fidelity_privacy_metrics.xlsx
@@ -1160,10 +1160,12 @@
           <t>CTGAN</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="C2" t="n">
+        <v>1.004611</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.9846819000000002</v>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>SDV</t>
@@ -1184,10 +1186,12 @@
           <t>CopulaGAN</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+      <c r="C3" t="n">
+        <v>1.072034</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.0012534</v>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>SDV</t>
@@ -1208,10 +1212,12 @@
           <t>TVAE</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>0.568466</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.4137232</v>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>SDV</t>
@@ -1232,10 +1238,12 @@
           <t>GaussianCopula</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="C5" t="n">
+        <v>0.232499</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.2147774</v>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>SDV</t>
@@ -2827,7 +2835,6 @@
           <t>Other_GAN</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0.037154</v>
       </c>
@@ -2858,7 +2865,6 @@
           <t>Other_GAN</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0.010063</v>
       </c>
@@ -2889,7 +2895,6 @@
           <t>Diffusion</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>0.424491</v>
       </c>
@@ -2920,7 +2925,6 @@
           <t>Diffusion</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0.012196</v>
       </c>

</xml_diff>